<commit_message>
Refine FSLR valuation framing and risk tracking
</commit_message>
<xml_diff>
--- a/outputs/first_solar_fslr_research_workbook_updated.xlsx
+++ b/outputs/first_solar_fslr_research_workbook_updated.xlsx
@@ -2,15 +2,15 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="1" r:id="R36bbfc4fd228421f"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Financials KPIs" sheetId="2" r:id="R761f0910782a4cad"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Valuation" sheetId="3" r:id="Rb42c5712f4d848a4"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Peers" sheetId="4" r:id="R3ec23ccfb4224443"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Market Reaction" sheetId="5" r:id="R913a6b2266bf4bb4"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Catalysts Policy Risks" sheetId="6" r:id="Rf654ab8705f140cc"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Research Path" sheetId="7" r:id="Re38465ecc3ee43d1"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sources" sheetId="8" r:id="R84dbae4f53fa4fa2"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Checks" sheetId="9" r:id="Rc55db5e070114ed8"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="1" r:id="Ra9d092ee60444485"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Financials KPIs" sheetId="2" r:id="Rb267487bad564653"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Valuation" sheetId="3" r:id="R4344cdc09e0846e2"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Peers" sheetId="4" r:id="R06291fd034054ad4"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Market Reaction" sheetId="5" r:id="Ra70283a520da4e8b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Catalysts Policy Risks" sheetId="6" r:id="Reb2fbfd51c50422f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Research Path" sheetId="7" r:id="R9d2e477346d34611"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sources" sheetId="8" r:id="R052bb57702a54759"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Checks" sheetId="9" r:id="R8f54c1f636414559"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -910,7 +910,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R3ea884af6f464916"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="Rd31962616f544dfd"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -940,7 +940,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="Rd5cb4642b17943ac"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="Rd54d5117c0f84d7b"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -975,7 +975,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R1bc16531c23a41c4"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="Rdc5d2b17e7a74fdf"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -1010,7 +1010,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R72212cc8143a4163"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="Rb06b8244902049fe"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -1045,7 +1045,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R403c550da548482e"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R4022620120f2445c"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -1126,8 +1126,8 @@
 </file>
 
 <file path=xl/tables/table4.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="4" name="CatalystsTable" displayName="CatalystsTable" ref="A4:H10" headerRowCount="1">
-  <x:autoFilter ref="A4:H10"/>
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="4" name="CatalystsTable" displayName="CatalystsTable" ref="A4:H11" headerRowCount="1">
+  <x:autoFilter ref="A4:H11"/>
   <x:tableColumns count="8">
     <x:tableColumn id="1" name="date_or_window"/>
     <x:tableColumn id="2" name="category"/>
@@ -1422,7 +1422,7 @@
         <x:v>投资方向</x:v>
       </x:c>
       <x:c r="B5" s="2" t="str">
-        <x:v>已有仓位继续跟踪；新资金等待回撤或订单/政策验证后分批</x:v>
+        <x:v>当前股价已接近基本面定价；继续持有更依赖 earnings power 兑现；新资金宜等待回撤、backlog ASP 改善、45X 政策确定性提高，或 2027-2029 收入桥更清晰</x:v>
       </x:c>
       <x:c r="C5" s="2"/>
       <x:c r="D5" s="2" t="str">
@@ -1448,7 +1448,7 @@
         <x:v>当前股价</x:v>
       </x:c>
       <x:c r="B6" s="8" t="n">
-        <x:v>297.895</x:v>
+        <x:v>297.74</x:v>
       </x:c>
       <x:c r="C6" s="2"/>
       <x:c r="D6" s="2" t="str">
@@ -1475,7 +1475,7 @@
       </x:c>
       <x:c r="B7" s="9" t="n">
         <x:f>Valuation!B9</x:f>
-        <x:v>30.057144424999994</x:v>
+        <x:v>30.040464099999998</x:v>
       </x:c>
       <x:c r="C7" s="2"/>
       <x:c r="D7" s="2" t="str">
@@ -1502,7 +1502,7 @@
       </x:c>
       <x:c r="B8" s="10" t="n">
         <x:f>Valuation!B15</x:f>
-        <x:v>11.13227571296296</x:v>
+        <x:v>11.126097814814813</x:v>
       </x:c>
       <x:c r="C8" s="2"/>
       <x:c r="D8" s="2" t="str">
@@ -1529,7 +1529,7 @@
       </x:c>
       <x:c r="B9" s="10" t="n">
         <x:f>Valuation!B13</x:f>
-        <x:v>19.243863049095605</x:v>
+        <x:v>19.233850129198963</x:v>
       </x:c>
       <x:c r="C9" s="2"/>
       <x:c r="D9" s="2"/>
@@ -1627,7 +1627,7 @@
       </x:c>
       <x:c r="F13" s="16" t="n">
         <x:f>E13/Valuation!$B$5-1</x:f>
-        <x:v>-0.3636270253686841</x:v>
+        <x:v>-0.3632957369591059</x:v>
       </x:c>
       <x:c r="G13" s="2"/>
       <x:c r="H13" s="2"/>
@@ -1654,7 +1654,7 @@
       </x:c>
       <x:c r="F14" s="16" t="n">
         <x:f>E14/Valuation!$B$5-1</x:f>
-        <x:v>-0.09536300596920877</x:v>
+        <x:v>-0.09489206241417847</x:v>
       </x:c>
       <x:c r="G14" s="2"/>
       <x:c r="H14" s="2"/>
@@ -1677,7 +1677,7 @@
       </x:c>
       <x:c r="F15" s="16" t="n">
         <x:f>E15/Valuation!$B$5-1</x:f>
-        <x:v>0.26024278718823535</x:v>
+        <x:v>0.26089885500584176</x:v>
       </x:c>
       <x:c r="G15" s="2"/>
       <x:c r="H15" s="2"/>
@@ -3694,7 +3694,7 @@
     <x:mergeCell ref="A2:H2"/>
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rf006ddbcc69b46c4"/>
+  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R79f367aa9ac54efc"/>
 </x:worksheet>
 </file>
 
@@ -6318,9 +6318,9 @@
     <x:mergeCell ref="A2:H2"/>
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R271846de203d4625"/>
+  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R3ce2eb04b5e84f6b"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rbb227ff90f524beb"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rddb0d529aeac4bbf"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -6432,7 +6432,7 @@
         <x:v>Current price</x:v>
       </x:c>
       <x:c r="B5" s="22" t="n">
-        <x:v>297.895</x:v>
+        <x:v>297.74</x:v>
       </x:c>
       <x:c r="C5" s="2" t="str">
         <x:v>USD/share</x:v>
@@ -6495,7 +6495,7 @@
       </x:c>
       <x:c r="B7" s="22" t="n">
         <x:f>B5*B6/1000</x:f>
-        <x:v>32.05797042499999</x:v>
+        <x:v>32.0412901</x:v>
       </x:c>
       <x:c r="C7" s="2" t="str">
         <x:v>USD bn</x:v>
@@ -6553,7 +6553,7 @@
       </x:c>
       <x:c r="B9" s="22" t="n">
         <x:f>B7-B8</x:f>
-        <x:v>30.057144424999994</x:v>
+        <x:v>30.040464099999998</x:v>
       </x:c>
       <x:c r="C9" s="2" t="str">
         <x:v>USD bn</x:v>
@@ -6658,7 +6658,7 @@
       </x:c>
       <x:c r="B13" s="22" t="n">
         <x:f>B5/B12</x:f>
-        <x:v>19.243863049095605</x:v>
+        <x:v>19.233850129198963</x:v>
       </x:c>
       <x:c r="C13" s="2" t="str">
         <x:v>x</x:v>
@@ -6685,7 +6685,7 @@
       </x:c>
       <x:c r="B14" s="22" t="n">
         <x:f>B9/B10</x:f>
-        <x:v>5.951909787128712</x:v>
+        <x:v>5.948606752475247</x:v>
       </x:c>
       <x:c r="C14" s="2" t="str">
         <x:v>x</x:v>
@@ -6712,7 +6712,7 @@
       </x:c>
       <x:c r="B15" s="22" t="n">
         <x:f>B9/B11</x:f>
-        <x:v>11.13227571296296</x:v>
+        <x:v>11.126097814814813</x:v>
       </x:c>
       <x:c r="C15" s="2" t="str">
         <x:v>x</x:v>
@@ -8828,7 +8828,7 @@
     <x:mergeCell ref="A2:H2"/>
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ra3607c1bcc484026"/>
+  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R7a5dfdb8ab104df1"/>
 </x:worksheet>
 </file>
 
@@ -8872,7 +8872,7 @@
     </x:row>
     <x:row r="2">
       <x:c r="A2" s="6" t="str">
-        <x:v>同行估值快照；FSLR 同时给出公司口径 cross-check。</x:v>
+        <x:v>Solar ecosystem directional comparison only; FSLR uses company-basis EV and deserves separate treatment because of CdTe, U.S. manufacturing, backlog and 45X sensitivity.</x:v>
       </x:c>
       <x:c r="B2" s="2"/>
       <x:c r="C2" s="2"/>
@@ -8974,16 +8974,16 @@
         <x:v>CdTe modules, U.S. manufacturing</x:v>
       </x:c>
       <x:c r="D5" s="30" t="n">
-        <x:v>297.895</x:v>
+        <x:v>297.74</x:v>
       </x:c>
       <x:c r="E5" s="30" t="n">
-        <x:v>31.89</x:v>
+        <x:v>32.04</x:v>
       </x:c>
       <x:c r="F5" s="30" t="n">
-        <x:v>27.57</x:v>
+        <x:v>30.04</x:v>
       </x:c>
       <x:c r="G5" s="30" t="n">
-        <x:v>19.17</x:v>
+        <x:v>19.23</x:v>
       </x:c>
       <x:c r="H5" s="30" t="n">
         <x:v>15.43</x:v>
@@ -8992,7 +8992,7 @@
         <x:v>5.43</x:v>
       </x:c>
       <x:c r="J5" s="30" t="n">
-        <x:v>5.09</x:v>
+        <x:v>5.54</x:v>
       </x:c>
       <x:c r="K5" s="30" t="n">
         <x:v>12.13</x:v>
@@ -9004,16 +9004,16 @@
         <x:v>S11</x:v>
       </x:c>
       <x:c r="N5" s="30" t="str">
-        <x:v>Secondary market data snapshot; FSLR valuation cross-checks also use company filings and guidance.</x:v>
+        <x:v>FSLR market cap/EV/PE use company-basis current price, Q1 diluted shares and Q1 net cash; peer multiples are directional only.</x:v>
       </x:c>
       <x:c r="O5" s="31" t="n">
-        <x:v>32.06</x:v>
+        <x:v>32.04</x:v>
       </x:c>
       <x:c r="P5" s="31" t="n">
-        <x:v>30.06</x:v>
+        <x:v>30.04</x:v>
       </x:c>
       <x:c r="Q5" s="31" t="n">
-        <x:v>19.24</x:v>
+        <x:v>19.23</x:v>
       </x:c>
       <x:c r="R5" s="29" t="n">
         <x:v>5.95</x:v>
@@ -9033,19 +9033,19 @@
         <x:v>microinverters/storage</x:v>
       </x:c>
       <x:c r="D6" s="30" t="n">
-        <x:v>71.01</x:v>
+        <x:v>72.15</x:v>
       </x:c>
       <x:c r="E6" s="30" t="n">
-        <x:v>9.39</x:v>
+        <x:v>9.48</x:v>
       </x:c>
       <x:c r="F6" s="30" t="n">
         <x:v>9.07</x:v>
       </x:c>
       <x:c r="G6" s="30" t="n">
-        <x:v>69.85</x:v>
+        <x:v>70.5</x:v>
       </x:c>
       <x:c r="H6" s="30" t="n">
-        <x:v>34.97</x:v>
+        <x:v>35.3</x:v>
       </x:c>
       <x:c r="I6" s="30" t="n">
         <x:v>6.71</x:v>
@@ -9063,7 +9063,7 @@
         <x:v>S11</x:v>
       </x:c>
       <x:c r="N6" s="30" t="str">
-        <x:v>Secondary market data snapshot; FSLR valuation cross-checks also use company filings and guidance.</x:v>
+        <x:v>Directional peer only: business model, margin structure, policy exposure and balance sheet differ from FSLR.</x:v>
       </x:c>
       <x:c r="O6" s="31" t="str"/>
       <x:c r="P6" s="31" t="str"/>
@@ -9082,17 +9082,17 @@
         <x:v>inverters/optimizer</x:v>
       </x:c>
       <x:c r="D7" s="30" t="n">
-        <x:v>74.125</x:v>
+        <x:v>74.255</x:v>
       </x:c>
       <x:c r="E7" s="30" t="n">
-        <x:v>4.52</x:v>
+        <x:v>4.51</x:v>
       </x:c>
       <x:c r="F7" s="30" t="n">
         <x:v>4.32</x:v>
       </x:c>
       <x:c r="G7" s="30" t="str"/>
       <x:c r="H7" s="30" t="n">
-        <x:v>123.19</x:v>
+        <x:v>126.2</x:v>
       </x:c>
       <x:c r="I7" s="30" t="n">
         <x:v>3.49</x:v>
@@ -9108,7 +9108,7 @@
         <x:v>S11</x:v>
       </x:c>
       <x:c r="N7" s="30" t="str">
-        <x:v>Secondary market data snapshot; FSLR valuation cross-checks also use company filings and guidance.</x:v>
+        <x:v>Directional peer only: business model, margin structure, policy exposure and balance sheet differ from FSLR.</x:v>
       </x:c>
       <x:c r="O7" s="31" t="str"/>
       <x:c r="P7" s="31" t="str"/>
@@ -9127,10 +9127,10 @@
         <x:v>modules/projects/storage</x:v>
       </x:c>
       <x:c r="D8" s="30" t="n">
-        <x:v>19.94</x:v>
+        <x:v>20.445</x:v>
       </x:c>
       <x:c r="E8" s="30" t="n">
-        <x:v>1.36</x:v>
+        <x:v>1.38</x:v>
       </x:c>
       <x:c r="F8" s="30" t="n">
         <x:v>6.93</x:v>
@@ -9153,7 +9153,7 @@
         <x:v>S11</x:v>
       </x:c>
       <x:c r="N8" s="30" t="str">
-        <x:v>Secondary market data snapshot; FSLR valuation cross-checks also use company filings and guidance.</x:v>
+        <x:v>Directional peer only: business model, margin structure, policy exposure and balance sheet differ from FSLR.</x:v>
       </x:c>
       <x:c r="O8" s="31" t="str"/>
       <x:c r="P8" s="31" t="str"/>
@@ -9172,10 +9172,10 @@
         <x:v>modules/global manufacturing</x:v>
       </x:c>
       <x:c r="D9" s="30" t="n">
-        <x:v>22.67</x:v>
+        <x:v>22.59</x:v>
       </x:c>
       <x:c r="E9" s="30" t="n">
-        <x:v>1.19</x:v>
+        <x:v>1.18</x:v>
       </x:c>
       <x:c r="F9" s="30" t="n">
         <x:v>4.17</x:v>
@@ -9198,7 +9198,7 @@
         <x:v>S11</x:v>
       </x:c>
       <x:c r="N9" s="30" t="str">
-        <x:v>Secondary market data snapshot; FSLR valuation cross-checks also use company filings and guidance.</x:v>
+        <x:v>Directional peer only: business model, margin structure, policy exposure and balance sheet differ from FSLR.</x:v>
       </x:c>
       <x:c r="O9" s="31" t="str"/>
       <x:c r="P9" s="31" t="str"/>
@@ -9217,17 +9217,17 @@
         <x:v>trackers</x:v>
       </x:c>
       <x:c r="D10" s="30" t="n">
-        <x:v>9.075</x:v>
+        <x:v>9.17</x:v>
       </x:c>
       <x:c r="E10" s="30" t="n">
-        <x:v>1.4</x:v>
+        <x:v>1.41</x:v>
       </x:c>
       <x:c r="F10" s="30" t="n">
         <x:v>1.95</x:v>
       </x:c>
       <x:c r="G10" s="30" t="str"/>
       <x:c r="H10" s="30" t="n">
-        <x:v>12.05</x:v>
+        <x:v>12.37</x:v>
       </x:c>
       <x:c r="I10" s="30" t="n">
         <x:v>1.15</x:v>
@@ -9245,7 +9245,7 @@
         <x:v>S11</x:v>
       </x:c>
       <x:c r="N10" s="30" t="str">
-        <x:v>Secondary market data snapshot; FSLR valuation cross-checks also use company filings and guidance.</x:v>
+        <x:v>Directional peer only: business model, margin structure, policy exposure and balance sheet differ from FSLR.</x:v>
       </x:c>
       <x:c r="O10" s="31" t="str"/>
       <x:c r="P10" s="31" t="str"/>
@@ -9267,16 +9267,16 @@
         <x:v>12.145</x:v>
       </x:c>
       <x:c r="E11" s="30" t="n">
-        <x:v>2.04</x:v>
+        <x:v>2.03</x:v>
       </x:c>
       <x:c r="F11" s="30" t="n">
         <x:v>2.25</x:v>
       </x:c>
       <x:c r="G11" s="30" t="n">
-        <x:v>60.18</x:v>
+        <x:v>60.83</x:v>
       </x:c>
       <x:c r="H11" s="30" t="n">
-        <x:v>26.17</x:v>
+        <x:v>26.45</x:v>
       </x:c>
       <x:c r="I11" s="30" t="n">
         <x:v>3.8</x:v>
@@ -9294,7 +9294,7 @@
         <x:v>S11</x:v>
       </x:c>
       <x:c r="N11" s="30" t="str">
-        <x:v>Secondary market data snapshot; FSLR valuation cross-checks also use company filings and guidance.</x:v>
+        <x:v>Directional peer only: business model, margin structure, policy exposure and balance sheet differ from FSLR.</x:v>
       </x:c>
       <x:c r="O11" s="31" t="str"/>
       <x:c r="P11" s="31" t="str"/>
@@ -9312,20 +9312,18 @@
       <x:c r="C12" s="20" t="str">
         <x:v>trackers/software</x:v>
       </x:c>
-      <x:c r="D12" s="30" t="n">
-        <x:v>134.8</x:v>
-      </x:c>
+      <x:c r="D12" s="30" t="str"/>
       <x:c r="E12" s="30" t="n">
-        <x:v>20.26</x:v>
+        <x:v>19.91</x:v>
       </x:c>
       <x:c r="F12" s="30" t="n">
         <x:v>19.08</x:v>
       </x:c>
       <x:c r="G12" s="30" t="n">
-        <x:v>35.11</x:v>
+        <x:v>34.49</x:v>
       </x:c>
       <x:c r="H12" s="30" t="n">
-        <x:v>29.09</x:v>
+        <x:v>28.58</x:v>
       </x:c>
       <x:c r="I12" s="30" t="n">
         <x:v>5.67</x:v>
@@ -9343,7 +9341,7 @@
         <x:v>S11</x:v>
       </x:c>
       <x:c r="N12" s="30" t="str">
-        <x:v>Secondary market data snapshot; FSLR valuation cross-checks also use company filings and guidance.</x:v>
+        <x:v>Directional peer only: business model, margin structure, policy exposure and balance sheet differ from FSLR.</x:v>
       </x:c>
       <x:c r="O12" s="31" t="str"/>
       <x:c r="P12" s="31" t="str"/>
@@ -9362,7 +9360,7 @@
         <x:v>residential solar/service</x:v>
       </x:c>
       <x:c r="D13" s="30" t="n">
-        <x:v>15.39</x:v>
+        <x:v>15.43</x:v>
       </x:c>
       <x:c r="E13" s="30" t="n">
         <x:v>3.67</x:v>
@@ -9371,10 +9369,10 @@
         <x:v>17.89</x:v>
       </x:c>
       <x:c r="G13" s="30" t="n">
-        <x:v>7.19</x:v>
+        <x:v>7.29</x:v>
       </x:c>
       <x:c r="H13" s="30" t="n">
-        <x:v>26.34</x:v>
+        <x:v>26.72</x:v>
       </x:c>
       <x:c r="I13" s="30" t="n">
         <x:v>1.16</x:v>
@@ -9392,7 +9390,7 @@
         <x:v>S11</x:v>
       </x:c>
       <x:c r="N13" s="30" t="str">
-        <x:v>Secondary market data snapshot; FSLR valuation cross-checks also use company filings and guidance.</x:v>
+        <x:v>Directional peer only: business model, margin structure, policy exposure and balance sheet differ from FSLR.</x:v>
       </x:c>
       <x:c r="O13" s="31" t="str"/>
       <x:c r="P13" s="31" t="str"/>
@@ -11460,7 +11458,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R45f0cde29fc246ce"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rc398bba2f762406a"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -13979,9 +13977,9 @@
     <x:mergeCell ref="A2:H2"/>
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Re8d349c39db54dea"/>
+  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R68d5cbb0bba54b67"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rb7490460d4b04c45"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R3a568eb4b4504fae"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -14252,28 +14250,28 @@
     </x:row>
     <x:row r="10">
       <x:c r="A10" s="20" t="str">
-        <x:v>Ongoing</x:v>
+        <x:v>2026-2029</x:v>
       </x:c>
       <x:c r="B10" s="20" t="str">
-        <x:v>Balance sheet</x:v>
+        <x:v>Execution / Demand</x:v>
       </x:c>
       <x:c r="C10" s="20" t="str">
-        <x:v>$1.5bn revolver and net cash</x:v>
+        <x:v>Backlog conversion and ASP durability</x:v>
       </x:c>
       <x:c r="D10" s="20" t="str">
-        <x:v>Strong liquidity</x:v>
+        <x:v>Core valuation driver</x:v>
       </x:c>
       <x:c r="E10" s="20" t="str">
-        <x:v>Net cash reduces downside and funds capacity; working capital swings can still move quarterly FCF.</x:v>
+        <x:v>Large backlog supports revenue visibility, but cancellations, delivery delays and lower new ASPs could weaken the 2027-2029 revenue bridge.</x:v>
       </x:c>
       <x:c r="F10" s="20" t="str">
-        <x:v>Net cash, revolver draw, operating cash flow and capex.</x:v>
+        <x:v>Net bookings GW, backlog ASP, cancellations, delivery schedule, customer concentration.</x:v>
       </x:c>
       <x:c r="G10" s="20" t="str">
-        <x:v>Low/Medium</x:v>
+        <x:v>High</x:v>
       </x:c>
       <x:c r="H10" s="20" t="str">
-        <x:v>S1;S2;S13</x:v>
+        <x:v>S1;S3;S4</x:v>
       </x:c>
       <x:c r="I10" s="2"/>
       <x:c r="J10" s="2"/>
@@ -14283,14 +14281,30 @@
       <x:c r="N10" s="2"/>
     </x:row>
     <x:row r="11">
-      <x:c r="A11" s="2"/>
-      <x:c r="B11" s="2"/>
-      <x:c r="C11" s="2"/>
-      <x:c r="D11" s="2"/>
-      <x:c r="E11" s="2"/>
-      <x:c r="F11" s="2"/>
-      <x:c r="G11" s="2"/>
-      <x:c r="H11" s="2"/>
+      <x:c r="A11" s="20" t="str">
+        <x:v>Ongoing</x:v>
+      </x:c>
+      <x:c r="B11" s="20" t="str">
+        <x:v>Balance sheet</x:v>
+      </x:c>
+      <x:c r="C11" s="20" t="str">
+        <x:v>$1.5bn revolver and net cash</x:v>
+      </x:c>
+      <x:c r="D11" s="20" t="str">
+        <x:v>Strong liquidity</x:v>
+      </x:c>
+      <x:c r="E11" s="20" t="str">
+        <x:v>Net cash reduces downside and funds capacity; working capital swings can still move quarterly FCF.</x:v>
+      </x:c>
+      <x:c r="F11" s="20" t="str">
+        <x:v>Net cash, revolver draw, operating cash flow and capex.</x:v>
+      </x:c>
+      <x:c r="G11" s="20" t="str">
+        <x:v>Low/Medium</x:v>
+      </x:c>
+      <x:c r="H11" s="20" t="str">
+        <x:v>S1;S2;S13</x:v>
+      </x:c>
       <x:c r="I11" s="2"/>
       <x:c r="J11" s="2"/>
       <x:c r="K11" s="2"/>
@@ -16369,7 +16383,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R7ffbfa6d09f544b3"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rc7e6fa87c74f49ae"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -16476,19 +16490,19 @@
     </x:row>
     <x:row r="5">
       <x:c r="A5" s="20" t="str">
-        <x:v>FSLR 现在贵不贵？</x:v>
+        <x:v>Is FSLR fairly valued, overvalued, or still underappreciated given 2026 EBITDA power and policy-adjusted risk?</x:v>
       </x:c>
       <x:c r="B5" s="20" t="str">
-        <x:v>当前股价已接近基本情景，继续上行要靠 earnings power 抬升或估值倍数扩张。</x:v>
+        <x:v>当前股价已接近基本面定价，继续上行要靠 earnings power 兑现、政策折现下降或估值倍数扩张。</x:v>
       </x:c>
       <x:c r="C5" s="20" t="str">
-        <x:v>FY2026 EBITDA midpoint vs actual run-rate; EV/FY2026 EBITDA; TTM EPS; net cash.</x:v>
+        <x:v>FY2026 EBITDA run-rate, EV/FY2026 EBITDA, TTM P/E, net cash, policy-adjusted multiple.</x:v>
       </x:c>
       <x:c r="D5" s="20" t="str">
         <x:v>EV/FY2026 EBITDA &lt;9x 且 backlog ASP 稳定更适合分批；&gt;11-12x 需要明确政策/订单催化。</x:v>
       </x:c>
       <x:c r="E5" s="20" t="str">
-        <x:v>约 11.1x EV/FY2026 EBITDA midpoint；接近基本情景。</x:v>
+        <x:v>At ~11.1x FY2026 EBITDA and ~19.2x TTM P/E, FSLR is no longer a deep-value solar trade; further upside needs gross margin strength, backlog conversion and policy clarity.</x:v>
       </x:c>
       <x:c r="F5" s="20" t="str">
         <x:v>S1;S3;S11;S12</x:v>
@@ -16507,16 +16521,16 @@
         <x:v>backlog 是护城河还是峰值订单？</x:v>
       </x:c>
       <x:c r="B6" s="20" t="str">
-        <x:v>47.9GW/$14.4bn 说明可见度强，但股票看的是新增订单价格和交付质量。</x:v>
+        <x:v>47.9GW/$14.4bn 说明可见度强，但股票看的是新增订单价格、取消风险和交付质量。</x:v>
       </x:c>
       <x:c r="C6" s="20" t="str">
-        <x:v>Net bookings GW, backlog value, backlog ASP, cancellations, delivery years.</x:v>
+        <x:v>Net bookings GW, new bookings ASP, backlog value, backlog ASP, cancellations, delivery years.</x:v>
       </x:c>
       <x:c r="D6" s="20" t="str">
         <x:v>新增 bookings ASP 接近或高于 $0.30/W，且 2027-2029 交付不断档。</x:v>
       </x:c>
       <x:c r="E6" s="20" t="str">
-        <x:v>Q1 后 backlog ASP 约 $0.30/W；YTD bookings 3.7GW。</x:v>
+        <x:v>Q1 后 backlog ASP 约 $0.30/W；YTD bookings 3.7GW；下一步必须验证新增订单 ASP。</x:v>
       </x:c>
       <x:c r="F6" s="20" t="str">
         <x:v>S1;S3</x:v>
@@ -16538,13 +16552,13 @@
         <x:v>45X 是 margin 和现金流的重要变量，政策折现率决定估值倍数。</x:v>
       </x:c>
       <x:c r="C7" s="20" t="str">
-        <x:v>45X recognized, cash realization, IRS/Treasury rules, PFE/FEOC restrictions.</x:v>
+        <x:v>45X recognized in gross profit, cash realization, tax-line treatment, IRS/Treasury rules, PFE/FEOC restrictions.</x:v>
       </x:c>
       <x:c r="D7" s="20" t="str">
         <x:v>规则稳定且公司披露现金化路径清晰，可降低市场折价。</x:v>
       </x:c>
       <x:c r="E7" s="20" t="str">
-        <x:v>FY2026 guide embeds about $2.145bn 45X credit；政策敏感度高。</x:v>
+        <x:v>FY2026 guide embeds about $2.145bn 45X credit；必须单独验证 cash realization，不能只看 EBITDA。</x:v>
       </x:c>
       <x:c r="F7" s="20" t="str">
         <x:v>S3;S6;S7</x:v>
@@ -16594,13 +16608,13 @@
         <x:v>增长股要从 capex 周期切到 FCF 周期才更容易重估。</x:v>
       </x:c>
       <x:c r="C9" s="20" t="str">
-        <x:v>Production GW, sold GW, capex, OCF, inventory, warranty, efficiency.</x:v>
+        <x:v>Production GW, sold GW, capex, OCF, inventory, warranty, efficiency, OCF-capex conversion.</x:v>
       </x:c>
       <x:c r="D9" s="20" t="str">
         <x:v>OCF &gt; capex 的季度持续出现，同时产能利用率上行。</x:v>
       </x:c>
       <x:c r="E9" s="20" t="str">
-        <x:v>2025 OCF $2.06bn，capex $0.87bn；Q1 2026 OCF 为负，仍有季节性和营运资本波动。</x:v>
+        <x:v>2025 OCF $2.06bn，capex $0.87bn；Q1 2026 OCF -$214.9mn，需跟踪 Q2/Q3 是否恢复。</x:v>
       </x:c>
       <x:c r="F9" s="20" t="str">
         <x:v>S2;S3;S4</x:v>
@@ -18717,7 +18731,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R5bead8a641a04497"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R55d2ee5a97e44f3f"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -21233,7 +21247,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rdbce0d0599ea481e"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R3585763771dd4c11"/>
   </x:tableParts>
 </x:worksheet>
 </file>

</xml_diff>